<commit_message>
KR RA5-10 → RA_single_600매 통합
</commit_message>
<xml_diff>
--- a/URL_LIST.xlsx
+++ b/URL_LIST.xlsx
@@ -559,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -582,7 +582,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GitHub Pages 호스팅 / 총 2000 unique 매 / 800 double + 1200 single = 2800 label slots</t>
+          <t>GitHub Pages 호스팅 / 총 2000 unique 매 / 800 double + 1200 single = 2800 label slots / KR 7 + JP 4 = 11 폴더</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>🇰🇷 KR (한국) — 12 폴더 / 1400 label slots / 1000 unique (400 double + 600 single)</t>
+          <t>🇰🇷 KR (한국) — 7 폴더 / 1400 label slots / 1000 unique (400 double + 600 single)</t>
         </is>
       </c>
     </row>
@@ -821,15 +821,15 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>RA_05_setE</t>
+          <t>RA_single_600매</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>단독 (chunk E)</t>
+          <t>단독 (chunks E~J 통합)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -840,318 +840,168 @@
       <c r="F12" s="10" t="inlineStr"/>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>https://sakie2000.github.io/labeling-packages/KR/RA_05_setE/</t>
+          <t>https://sakie2000.github.io/labeling-packages/KR/RA_single_600매/</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="13" t="n">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>KR 소계: 사키에 2 폴더 (400 labels) + RA paired 4 폴더 (400 labels) + RA single 1 폴더 600매 = 1400 labels / 1000 unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>🇯🇵 JP (일본) — 4 폴더 / 1400 label slots / 1000 unique (400 double + 600 single)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>RA_06_setF</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>단독 (chunk F)</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>RA6</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr"/>
-      <c r="G13" s="14" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/KR/RA_06_setF/</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="inlineStr"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>RA_07_setG</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>단독 (chunk G)</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>RA7</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr"/>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/KR/RA_07_setG/</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>RA_08_setH</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>단독 (chunk H)</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>RA8</t>
-        </is>
-      </c>
-      <c r="F15" s="14" t="inlineStr"/>
-      <c r="G15" s="14" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/KR/RA_08_setH/</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>RA_09_setI</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>단독 (chunk I)</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>RA9</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr"/>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/KR/RA_09_setI/</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr"/>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>사키에_JP_200매</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>단독 (사키에)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>사키에</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>https://sakie2000.github.io/labeling-packages/JP/사키에_JP_200매/</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>RA_10_setJ</t>
+          <t>나츠미_400매</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>단독 (chunk J)</t>
+          <t>단독 (나츠미)</t>
         </is>
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>RA10</t>
+          <t>나츠미</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr"/>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>https://sakie2000.github.io/labeling-packages/KR/RA_10_setJ/</t>
+          <t>https://sakie2000.github.io/labeling-packages/JP/나츠미_400매/</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>KR 소계: 사키에 2 폴더 (400 labels) + RA paired 4 폴더 (400 labels) + RA single 6 폴더 (600 labels) = 1400 labels / 1000 unique</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>🇯🇵 JP (일본) — 4 폴더 / 1400 label slots / 1000 unique (400 double + 600 single)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>사키에_JP_200매</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>단독 (사키에)</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>사키에</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr"/>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/JP/사키에_JP_200매/</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>나츠미_400매</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="n">
+      <c r="A18" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>RA_c_400매</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>단독 (나츠미)</t>
-        </is>
-      </c>
-      <c r="E22" s="16" t="inlineStr">
-        <is>
-          <t>나츠미</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr"/>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/JP/나츠미_400매/</t>
-        </is>
-      </c>
-      <c r="H22" s="15" t="inlineStr"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>RA_c_400매</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>RA_d 와 同 (double)</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>코이미</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr"/>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>https://sakie2000.github.io/labeling-packages/JP/RA_c_400매/</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>RA_d_400매</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="D23" s="10" t="inlineStr">
-        <is>
-          <t>RA_d 와 同 (double)</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>코이미</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr"/>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>https://sakie2000.github.io/labeling-packages/JP/RA_c_400매/</t>
-        </is>
-      </c>
-      <c r="H23" s="11" t="inlineStr"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>RA_d_400매</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="n">
-        <v>400</v>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>RA_c 와 同 (double)</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>가야</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr"/>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="F19" s="14" t="inlineStr"/>
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>https://sakie2000.github.io/labeling-packages/JP/RA_d_400매/</t>
         </is>
       </c>
-      <c r="H24" s="15" t="inlineStr"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="H19" s="15" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>JP 소계: 사키에 200 + 나츠미 400 + RA_c (코이미) 400 + RA_d (가야) 400 = 1400 labels / 1000 unique</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>📊 전체: 2000 unique 매 / 2800 label slots (800 double + 1200 single) | 발급 URL: 13 개 (사키에 폴더 3 개는 본인 사용 OK)</t>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>📊 전체: 2000 unique 매 / 2800 label slots (800 double + 1200 single) | 발급 URL: 8 개 (사키에 폴더 3 개는 본인 사용 OK)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1325,7 +1175,7 @@
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>1. KR 10 RA 모집·연락처 확보 (paired 4 + single 6)</t>
+          <t>1. KR 5 RA 모집·연락처 확보 (paired 4 + single 1 × 600매)</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1211,7 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>4. 각 라벨러에 카톡 송신 (13 URL)</t>
+          <t>4. 각 라벨러에 카톡 송신 (8 URL)</t>
         </is>
       </c>
     </row>

</xml_diff>